<commit_message>
feat: inicializar estructura base, clase Cliente y logs de errores
</commit_message>
<xml_diff>
--- a/matriz_trabajo_equipo_programacion.xlsx
+++ b/matriz_trabajo_equipo_programacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fredy Tangarife\Documents\INGENIERIA DE SISTEMAS UNAD\Semestre 2026-1\PROGRAMACION\FASE 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{136EBC44-75A8-4566-805D-79DF4A85EDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66A45A6-8ED5-4492-BE54-E1CEBB9C2BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B3ACD2CA-97D0-4560-84EB-280C7D8F55A1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>Nombre del estudiante</t>
   </si>
@@ -56,19 +56,150 @@
   </si>
   <si>
     <t>Estado</t>
+  </si>
+  <si>
+    <t>Planificación</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>Luis David Gomez Pinto</t>
+  </si>
+  <si>
+    <t>Jose Gabriel Castro Lopez</t>
+  </si>
+  <si>
+    <t>Juan Esteban Cardenas Alvarez</t>
+  </si>
+  <si>
+    <t>Diyein Erlency Botero Betancourt</t>
+  </si>
+  <si>
+    <t>Fase: Control de Errores y Logs
+Excepciones Propias: Crear clases como DatosInvalidosError y ServicioNoDisponibleError.
+Sistema de Logs: Configurar el archivo .txt para que registre automáticamente cada evento o fallo del sistema.</t>
+  </si>
+  <si>
+    <t>Fredy Andres Tangarife Correa</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Fase:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Cimientos y Datos. 
+Crear Clase Abstracta EntidadGeneral. Definir el método mostrar_detalles.
+Crear Clase Cliente: Atributos privados (__nombre, __documento), validaciones de correo/texto y uso de @property.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Fase: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Catálogo de Servicios
+Crear Clase Abstracta Servicio: Atributos de ID, nombre y costo base. Crear Subclases (Herencia): Crear ReservaSala, AlquilerEquipo y AsesoriaEspecializada.
+Polimorfismo: Sobrescribir calcular_costo con lógica distinta para cada una.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Fase:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Lógica de Negocio
+Crear Clase Reserva: Relacionar Cliente con Servicio y duración.
+Manejo de Excepciones: Implementar confirmar() usando la estructura completa try/except/else/finally para validar disponibilidad y costos.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Fase: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Integración y Pruebas
+Gestión en Memoria: Crear las listas de clientes, servicios y reservas en el main.py.
+Simulación: Programar las 10 operaciones (exitosas y fallidas) asegurando que el programa no se detenga si ocurre un error grave.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -79,7 +210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -87,12 +218,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,30 +573,149 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173896AA-BE34-452E-8E58-A3BA00C337BD}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="21.7109375" style="4"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" ht="210" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E2" s="8">
+        <v>46137</v>
+      </c>
+      <c r="F2" s="6">
+        <v>10</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" ht="255" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E3" s="8">
+        <v>46137</v>
+      </c>
+      <c r="F3" s="6">
+        <v>10</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="2" customFormat="1" ht="225" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E4" s="8">
+        <v>46137</v>
+      </c>
+      <c r="F4" s="6">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="2" customFormat="1" ht="210" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E5" s="8">
+        <v>46137</v>
+      </c>
+      <c r="F5" s="6">
+        <v>10</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" ht="210" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E6" s="8">
+        <v>46137</v>
+      </c>
+      <c r="F6" s="6">
+        <v>10</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>